<commit_message>
docuemntacion y codigo actualizado
</commit_message>
<xml_diff>
--- a/instagram_masivo.xlsx
+++ b/instagram_masivo.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instagram Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,8 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -442,6 +447,11 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
@@ -449,83 +459,85 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>marvel</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>11122</v>
-      </c>
-      <c r="C2" t="n">
-        <v>64500000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>197</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>46134.92010451053</v>
+          <t>masa</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:34:54</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>instagram</t>
+          <t>nike</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8411</v>
+        <v>1630</v>
       </c>
       <c r="C3" t="n">
-        <v>700000000</v>
+        <v>297</v>
       </c>
       <c r="D3" t="n">
-        <v>246</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>46134.92010451289</v>
+        <v>240</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:34:54</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fcbarcelona</t>
+          <t>marvellatam</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26977</v>
+        <v>4374</v>
       </c>
       <c r="C4" t="n">
-        <v>147000000</v>
+        <v>39</v>
       </c>
       <c r="D4" t="n">
-        <v>107</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>46134.9201045134</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>lahoraec</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>46134.92010451375</v>
+        <v>33</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-04-28 19:34:54</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>